<commit_message>
Add management command to import term 3 balances
</commit_message>
<xml_diff>
--- a/active_students_balances.xlsx
+++ b/active_students_balances.xlsx
@@ -1948,7 +1948,7 @@
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
@@ -6618,6 +6618,9 @@
       </c>
       <c r="B568" s="0" t="n">
         <v>-500</v>
+      </c>
+      <c r="C568" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="569" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>